<commit_message>
Update combined Excel files with new data
</commit_message>
<xml_diff>
--- a/combined_excel_from_all_sheets.xlsx
+++ b/combined_excel_from_all_sheets.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -573,111 +573,101 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_1</t>
+          <t>MFA_Template_sorting_flow_2_PP</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Mixed Plastics</t>
+          <t>PP in PP sorted products</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Flm material (mostly based on LDPE)</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>83,292.6 Mg/a ± 45.2%</t>
-        </is>
+          <t>PP food packaging</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>21.2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_1</t>
+          <t>MFA_Template_sorting_flow_2_PP</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mixed Plastics</t>
+          <t>PP in PP sorted products</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>HDPE</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>92,958.3 Mg/a ± 8.0%</t>
-        </is>
+          <t>Mix food packaging</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>10.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_1</t>
+          <t>MFA_Template_sorting_flow_2_PP</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Mixed Plastics</t>
+          <t>PP in PP sorted products</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>PP</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>109,442.7 Mg/a ± 7.8%</t>
-        </is>
+          <t>PE non-food packaging</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_1</t>
+          <t>MFA_Template_sorting_flow_2_PP</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mixed Plastics</t>
+          <t>PP in PP sorted products</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>17,744.6 Mg/a ± 30.8%</t>
-        </is>
+          <t>PP non-food packaging</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>12.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_1</t>
+          <t>MFA_Template_sorting_flow_2_PP</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Mixed Plastics</t>
+          <t>PP in PP sorted products</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>PET</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>52,529.6 Mg/a ± 11.9%</t>
-        </is>
+          <t>PP trays</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>3.8</v>
       </c>
     </row>
     <row r="13">
@@ -693,11 +683,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PP food packaging</t>
+          <t>Black plastics</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>21.2</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -713,11 +703,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Mix food packaging</t>
+          <t>Foils ≥ DIN A4</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>10.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -733,11 +723,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PE non-food packaging</t>
+          <t>Foils &lt; DIN A4</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1.1</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="16">
@@ -753,11 +743,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PP non-food packaging</t>
+          <t>Non Packaging Plastics</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>12.1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17">
@@ -773,11 +763,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PP trays</t>
+          <t>Packaging Composites</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3.8</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="18">
@@ -793,11 +783,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Black plastics</t>
+          <t>Residues coarse</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="19">
@@ -813,11 +803,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Foils ≥ DIN A4</t>
+          <t>Fine &lt; 40 mm</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="20">
@@ -833,67 +823,69 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Foils &lt; DIN A4</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>5.3</v>
+          <t>Moisture and dirt</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>15.4% ± 11.0%</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PP</t>
+          <t>MFA_Template_sorting_flow_2_PS</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PP in PP sorted products</t>
+          <t>PS in PS sorted products</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Non Packaging Plastics</t>
+          <t>Mix food packaging</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>17</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PP</t>
+          <t>MFA_Template_sorting_flow_2_PS</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PP in PP sorted products</t>
+          <t>PS in PS sorted products</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Packaging Composites</t>
+          <t>PS rigids</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1.3</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PP</t>
+          <t>MFA_Template_sorting_flow_2_PS</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PP in PP sorted products</t>
+          <t>PS in PS sorted products</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Residues coarse</t>
+          <t>EPS</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -903,43 +895,41 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PP</t>
+          <t>MFA_Template_sorting_flow_2_PS</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PP in PP sorted products</t>
+          <t>PS in PS sorted products</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Fine &lt; 40 mm</t>
+          <t>PP non-food packaging</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>4.7</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PP</t>
+          <t>MFA_Template_sorting_flow_2_PS</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PP in PP sorted products</t>
+          <t>PS in PS sorted products</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Moisture and dirt</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>15.4% ± 11.0%</t>
-        </is>
+          <t>Black plastics</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1.7</v>
       </c>
     </row>
     <row r="26">
@@ -955,11 +945,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mix food packaging</t>
+          <t>Non Packaging Plastics</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1.9</v>
+        <v>32.7</v>
       </c>
     </row>
     <row r="27">
@@ -975,11 +965,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PS rigids</t>
+          <t>Fine &lt; 40 mm</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>42.5</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="28">
@@ -995,113 +985,113 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>EPS</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>1.2</v>
+          <t>Moisture and dirt</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>12.4% ± 9.9%</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PS</t>
+          <t>MFA_Template_sorting_flow_2_PET</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PS in PS sorted products</t>
+          <t>PET in PET sorted products</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PP non-food packaging</t>
+          <t>PET food packaging clear</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>12.1</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PS</t>
+          <t>MFA_Template_sorting_flow_2_PET</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PS in PS sorted products</t>
+          <t>PET in PET sorted products</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Black plastics</t>
+          <t>PET food packaging coloured</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1.7</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PS</t>
+          <t>MFA_Template_sorting_flow_2_PET</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PS in PS sorted products</t>
+          <t>PET in PET sorted products</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Non Packaging Plastics</t>
+          <t>Mix food packaginga</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>32.7</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PS</t>
+          <t>MFA_Template_sorting_flow_2_PET</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PS in PS sorted products</t>
+          <t>PET in PET sorted products</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Fine &lt; 40 mm</t>
+          <t>PET non-food packaging</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2.9</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PS</t>
+          <t>MFA_Template_sorting_flow_2_PET</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PS in PS sorted products</t>
+          <t>PET in PET sorted products</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Moisture and dirt</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>12.4% ± 9.9%</t>
-        </is>
+          <t>PET trays</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="34">
@@ -1117,11 +1107,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PET food packaging clear</t>
+          <t>Black plastics</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>19.1</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="35">
@@ -1137,11 +1127,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>PET food packaging coloured</t>
+          <t>Foils &lt; DIN A4</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5.2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="36">
@@ -1157,11 +1147,11 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Mix food packaginga</t>
+          <t>Non Packaging Plastics</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>17.5</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="37">
@@ -1177,11 +1167,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PET non-food packaging</t>
+          <t>Packaging Composites</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>15.8</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="38">
@@ -1197,11 +1187,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PET trays</t>
+          <t>Fine &lt; 40 mm</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>17</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="39">
@@ -1217,113 +1207,113 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Black plastics</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>1.6</v>
+          <t>Moisture and dirt</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>11.4% ± 3.8%</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PET</t>
+          <t>MFA_Template_sorting_flow_2_HDP</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PET in PET sorted products</t>
+          <t>HDPE in HDPE sorted products</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Foils &lt; DIN A4</t>
+          <t>PE food packaging</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1.5</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PET</t>
+          <t>MFA_Template_sorting_flow_2_HDP</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PET in PET sorted products</t>
+          <t>HDPE in HDPE sorted products</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Non Packaging Plastics</t>
+          <t>PE non-food packaging</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>2.4</v>
+        <v>62.6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PET</t>
+          <t>MFA_Template_sorting_flow_2_HDP</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PET in PET sorted products</t>
+          <t>HDPE in HDPE sorted products</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Packaging Composites</t>
+          <t>Black plastics</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PET</t>
+          <t>MFA_Template_sorting_flow_2_HDP</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PET in PET sorted products</t>
+          <t>HDPE in HDPE sorted products</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Fine &lt; 40 mm</t>
+          <t>Foils &lt; DIN A4</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_PET</t>
+          <t>MFA_Template_sorting_flow_2_HDP</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PET in PET sorted products</t>
+          <t>HDPE in HDPE sorted products</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Moisture and dirt</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>11.4% ± 3.8%</t>
-        </is>
+          <t>Non Packaging Plastics</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>12.4</v>
       </c>
     </row>
     <row r="45">
@@ -1339,11 +1329,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PE food packaging</t>
+          <t>Packaging Composites</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>6.4</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="46">
@@ -1359,11 +1349,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PE non-food packaging</t>
+          <t>Fine &lt; 40 mm</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>62.6</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="47">
@@ -1379,102 +1369,104 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Black plastics</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
-        <v>2.3</v>
+          <t>Moisture and dirt</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>6.8% ± 3.1%</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_HDP</t>
+          <t>MFA_Template_sorting_flow_2_Fil</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>HDPE in HDPE sorted products</t>
+          <t>Film in film sorted products</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Foils &lt; DIN A4</t>
+          <t>Black plastics</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>2.5</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_HDP</t>
+          <t>MFA_Template_sorting_flow_2_Fil</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>HDPE in HDPE sorted products</t>
+          <t>Film in film sorted products</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Non Packaging Plastics</t>
+          <t>Foils ≥ DIN A4</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>12.4</v>
+        <v>46.6</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_HDP</t>
+          <t>MFA_Template_sorting_flow_2_Fil</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>HDPE in HDPE sorted products</t>
+          <t>Film in film sorted products</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Packaging Composites</t>
+          <t>Foils &lt; DIN A4</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1.1</v>
+        <v>23.2</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_HDP</t>
+          <t>MFA_Template_sorting_flow_2_Fil</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>HDPE in HDPE sorted products</t>
+          <t>Film in film sorted products</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Fine &lt; 40 mm</t>
+          <t>Non Packaging Plastics</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>2.5</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MFA_Template_sorting_flow_2_HDP</t>
+          <t>MFA_Template_sorting_flow_2_Fil</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>HDPE in HDPE sorted products</t>
+          <t>Film in film sorted products</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1483,108 +1475,6 @@
         </is>
       </c>
       <c r="D52" t="inlineStr">
-        <is>
-          <t>6.8% ± 3.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>MFA_Template_sorting_flow_2_Fil</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Film in film sorted products</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Black plastics</t>
-        </is>
-      </c>
-      <c r="D53" t="n">
-        <v>1.1</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>MFA_Template_sorting_flow_2_Fil</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Film in film sorted products</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Foils ≥ DIN A4</t>
-        </is>
-      </c>
-      <c r="D54" t="n">
-        <v>46.6</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>MFA_Template_sorting_flow_2_Fil</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Film in film sorted products</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Foils &lt; DIN A4</t>
-        </is>
-      </c>
-      <c r="D55" t="n">
-        <v>23.2</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>MFA_Template_sorting_flow_2_Fil</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Film in film sorted products</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Non Packaging Plastics</t>
-        </is>
-      </c>
-      <c r="D56" t="n">
-        <v>3.8</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>MFA_Template_sorting_flow_2_Fil</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Film in film sorted products</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Moisture and dirt</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
         <is>
           <t>19.8% ± 6.9%</t>
         </is>

</xml_diff>